<commit_message>
Ignore XLSX and result.md; update Step 12 selection logic and file-open behavior
</commit_message>
<xml_diff>
--- a/family_tree_highlighted.xlsx
+++ b/family_tree_highlighted.xlsx
@@ -62,10 +62,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1782,7 +1782,7 @@
           <t>9411</t>
         </is>
       </c>
-      <c r="M17" s="1" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>9941</t>
         </is>
@@ -2558,7 +2558,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>7440</t>
         </is>
@@ -2935,7 +2935,7 @@
           <t>9100</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>9110</t>
         </is>
@@ -3010,7 +3010,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>9110</t>
         </is>
@@ -3978,7 +3978,7 @@
           <t>7740</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" s="1" t="inlineStr">
         <is>
           <t>7440</t>
         </is>
@@ -4093,7 +4093,7 @@
           <t>7750</t>
         </is>
       </c>
-      <c r="M46" s="1" t="inlineStr">
+      <c r="M46" s="3" t="inlineStr">
         <is>
           <t>7550</t>
         </is>

</xml_diff>